<commit_message>
Feature Update: 1) combining role of both Facilitator and Summarizer to a single facilitator role, 2) Allow profile to be build using Q&A format, backstories, both or none; 3) Remove API keys from being printed during experiment verification and allow package version to be printed; 4) Allow users to define roles and treatments using a Python dictionary and these attributes can be accessed using Jjinja dot notation in the prompt worksheet; 5) Users have full control over where and when the treatment arm is introduced; 6) Introduce support for repeated rounds for private and public questions and control flow functionality; 7) Introduce support for OpenRouter.ai APIs.
</commit_message>
<xml_diff>
--- a/demos/prompt_template.xlsx
+++ b/demos/prompt_template.xlsx
@@ -1,27 +1,27 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11003"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11102"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/raymondlow/Documents/talking-to-machines/talking-to-machines/demos/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{180DC00D-0321-CD4F-A62A-457C5D856094}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AAC41F47-255B-584E-9FD4-DC9AE09E0AC3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="3700" yWindow="760" windowWidth="30860" windowHeight="20140" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="3620" yWindow="3400" windowWidth="34560" windowHeight="20140" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="experimental_setting" sheetId="1" r:id="rId1"/>
-    <sheet name="treatments" sheetId="2" r:id="rId2"/>
-    <sheet name="roles" sheetId="3" r:id="rId3"/>
-    <sheet name="interview_prompts" sheetId="4" r:id="rId4"/>
-    <sheet name="demographic_profiles" sheetId="5" r:id="rId5"/>
-    <sheet name="constants" sheetId="6" r:id="rId6"/>
+    <sheet name="settings" sheetId="1" r:id="rId1"/>
+    <sheet name="treatment" sheetId="2" r:id="rId2"/>
+    <sheet name="role" sheetId="3" r:id="rId3"/>
+    <sheet name="prompt" sheetId="4" r:id="rId4"/>
+    <sheet name="profile" sheetId="5" r:id="rId5"/>
+    <sheet name="constant" sheetId="6" r:id="rId6"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">demographic_profiles!$A$1:$Y$5312</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">profile!$A$1:$Y$5312</definedName>
   </definedNames>
   <calcPr calcId="0"/>
   <extLst>
@@ -33,30 +33,15 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="43" uniqueCount="39">
-  <si>
-    <t>experimental_setting</t>
-  </si>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="46" uniqueCount="40">
   <si>
     <t>value</t>
-  </si>
-  <si>
-    <t>experiment_id</t>
   </si>
   <si>
     <t>model_info</t>
   </si>
   <si>
-    <t>num_sessions</t>
-  </si>
-  <si>
-    <t>max_conversation_length</t>
-  </si>
-  <si>
     <t>treatment_assignment_strategy</t>
-  </si>
-  <si>
-    <t>session_assignment_strategy</t>
   </si>
   <si>
     <t>role_assignment_strategy</t>
@@ -65,22 +50,10 @@
     <t>treatment_label</t>
   </si>
   <si>
-    <t>treatment_description</t>
-  </si>
-  <si>
     <t>role_label</t>
   </si>
   <si>
-    <t>role_description</t>
-  </si>
-  <si>
-    <t>task_id</t>
-  </si>
-  <si>
     <t>type</t>
-  </si>
-  <si>
-    <t>task_order</t>
   </si>
   <si>
     <t>is_adapted</t>
@@ -90,12 +63,6 @@
   </si>
   <si>
     <t>llm_text</t>
-  </si>
-  <si>
-    <t>var_name</t>
-  </si>
-  <si>
-    <t>var_type</t>
   </si>
   <si>
     <t>response_options</t>
@@ -110,13 +77,7 @@
     <t>generate_speculation_score</t>
   </si>
   <si>
-    <t>name</t>
-  </si>
-  <si>
     <t>random_seed</t>
-  </si>
-  <si>
-    <t>session_column</t>
   </si>
   <si>
     <t>role_column</t>
@@ -131,25 +92,69 @@
     <t>format_response</t>
   </si>
   <si>
-    <t>include_backstories</t>
-  </si>
-  <si>
     <t>hf_inference_endpoint</t>
-  </si>
-  <si>
-    <t>Assume the role of a facilitator in an experiment.</t>
-  </si>
-  <si>
-    <t>Facilitator</t>
-  </si>
-  <si>
-    <t>num_subjects_per_session</t>
   </si>
   <si>
     <t>context</t>
   </si>
   <si>
     <t>Provide the context of the experiment here</t>
+  </si>
+  <si>
+    <t>settings_label</t>
+  </si>
+  <si>
+    <t>session_id</t>
+  </si>
+  <si>
+    <t>num_subjects_per_group</t>
+  </si>
+  <si>
+    <t>num_groups</t>
+  </si>
+  <si>
+    <t>group_assignment_strategy</t>
+  </si>
+  <si>
+    <t>group_column</t>
+  </si>
+  <si>
+    <t>build_profile_qna</t>
+  </si>
+  <si>
+    <t>build_profile_backstories</t>
+  </si>
+  <si>
+    <t>{
+"description":"Assume the role of a facilitator in an experiment."
+}</t>
+  </si>
+  <si>
+    <t>facilitator</t>
+  </si>
+  <si>
+    <t>constant_label</t>
+  </si>
+  <si>
+    <t>round_id</t>
+  </si>
+  <si>
+    <t>round_order</t>
+  </si>
+  <si>
+    <t>response_name</t>
+  </si>
+  <si>
+    <t>response_type</t>
+  </si>
+  <si>
+    <t>ID</t>
+  </si>
+  <si>
+    <t>subject_id</t>
+  </si>
+  <si>
+    <t>max_num_rounds</t>
   </si>
 </sst>
 </file>
@@ -196,7 +201,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -208,6 +213,9 @@
     </xf>
     <xf numFmtId="22" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
   </cellXfs>
@@ -435,69 +443,69 @@
   <sheetData>
     <row r="1" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="B1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
+    </row>
+    <row r="2" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A2" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="B2" s="1"/>
+    </row>
+    <row r="3" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A3" s="1" t="s">
         <v>1</v>
       </c>
-    </row>
-    <row r="2" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A2" s="1" t="s">
+      <c r="B3" s="1"/>
+    </row>
+    <row r="4" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A4" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="B4" s="1"/>
+    </row>
+    <row r="5" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A5" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="B5" s="1"/>
+    </row>
+    <row r="6" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A6" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="B6" s="2"/>
+    </row>
+    <row r="7" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A7" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="B7" s="2"/>
+    </row>
+    <row r="8" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A8" s="1" t="s">
+        <v>39</v>
+      </c>
+      <c r="B8" s="2"/>
+    </row>
+    <row r="9" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A9" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="B2" s="1"/>
-    </row>
-    <row r="3" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A3" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="B3" s="1"/>
-    </row>
-    <row r="4" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A4" s="1" t="s">
-        <v>33</v>
-      </c>
-      <c r="B4" s="1"/>
-    </row>
-    <row r="5" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A5" s="1" t="s">
-        <v>30</v>
-      </c>
-      <c r="B5" s="1"/>
-    </row>
-    <row r="6" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A6" s="1" t="s">
-        <v>36</v>
-      </c>
-      <c r="B6" s="2"/>
-    </row>
-    <row r="7" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A7" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="B7" s="2"/>
-    </row>
-    <row r="8" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A8" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="B8" s="2"/>
-    </row>
-    <row r="9" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A9" s="1" t="s">
-        <v>6</v>
-      </c>
       <c r="B9" s="1"/>
     </row>
     <row r="10" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A10" s="1" t="s">
-        <v>29</v>
+        <v>16</v>
       </c>
       <c r="B10" s="1"/>
     </row>
     <row r="11" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A11" s="1" t="s">
-        <v>7</v>
+        <v>26</v>
       </c>
       <c r="B11" s="1"/>
     </row>
@@ -509,40 +517,44 @@
     </row>
     <row r="13" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A13" s="3" t="s">
-        <v>8</v>
+        <v>3</v>
       </c>
     </row>
     <row r="14" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A14" s="3" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="15" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A15" s="3" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="16" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A16" s="3" t="s">
         <v>28</v>
       </c>
     </row>
-    <row r="15" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A15" s="3" t="s">
-        <v>26</v>
+    <row r="17" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A17" s="3" t="s">
+        <v>29</v>
       </c>
     </row>
-    <row r="16" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A16" s="3" t="s">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="17" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="18" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="19" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="20" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="21" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="22" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="23" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="24" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="25" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="26" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="27" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="28" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="29" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="30" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="31" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="32" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="18" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="19" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="20" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="21" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="22" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="23" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="24" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="25" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="26" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="27" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="28" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="29" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="30" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="31" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="32" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
     <row r="33" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
     <row r="34" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
     <row r="35" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
@@ -1531,7 +1543,7 @@
     <dataValidation type="list" allowBlank="1" showErrorMessage="1" errorTitle="Invalid Value" error="Please choose a role assignment strategy from the dropdown list." sqref="B13" xr:uid="{CD5A8A2F-647C-7140-A110-46420E7F8C2F}">
       <formula1>"random, manual"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showErrorMessage="1" errorTitle="Invalid Value" error="Please choose an option from the dropdown list." sqref="B16" xr:uid="{E2415674-B0C6-6543-8726-22265FD96C3A}">
+    <dataValidation type="list" allowBlank="1" showErrorMessage="1" errorTitle="Invalid Value" error="Please choose an option from the dropdown list." sqref="B16:B17" xr:uid="{E2415674-B0C6-6543-8726-22265FD96C3A}">
       <formula1>"True, False"</formula1>
     </dataValidation>
   </dataValidations>
@@ -1545,17 +1557,18 @@
   <dimension ref="A1:B1000"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="11.1640625" defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="2" width="14.1640625" style="3" customWidth="1"/>
+    <col min="1" max="1" width="15.33203125" style="3" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="14.1640625" style="3" customWidth="1"/>
     <col min="3" max="27" width="10.6640625" style="3" customWidth="1"/>
     <col min="28" max="16384" width="11.1640625" style="3"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
-        <v>9</v>
+        <v>4</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>10</v>
+        <v>0</v>
       </c>
     </row>
     <row r="2" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
@@ -2586,18 +2599,18 @@
   <sheetData>
     <row r="1" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
-        <v>11</v>
+        <v>5</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>12</v>
+        <v>0</v>
       </c>
     </row>
     <row r="2" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A2" s="1" t="s">
-        <v>35</v>
+        <v>31</v>
       </c>
       <c r="B2" s="4" t="s">
-        <v>34</v>
+        <v>30</v>
       </c>
     </row>
     <row r="3" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
@@ -3623,43 +3636,43 @@
   <sheetData>
     <row r="1" spans="1:13" ht="16.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A1" s="3" t="s">
+        <v>33</v>
+      </c>
+      <c r="B1" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="C1" s="3" t="s">
+        <v>34</v>
+      </c>
+      <c r="D1" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="E1" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="F1" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="G1" s="3" t="s">
+        <v>35</v>
+      </c>
+      <c r="H1" s="3" t="s">
+        <v>36</v>
+      </c>
+      <c r="I1" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="J1" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="K1" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="L1" s="3" t="s">
         <v>13</v>
       </c>
-      <c r="B1" s="3" t="s">
-        <v>14</v>
-      </c>
-      <c r="C1" s="3" t="s">
-        <v>15</v>
-      </c>
-      <c r="D1" s="3" t="s">
-        <v>16</v>
-      </c>
-      <c r="E1" s="3" t="s">
-        <v>17</v>
-      </c>
-      <c r="F1" s="3" t="s">
+      <c r="M1" s="3" t="s">
         <v>18</v>
-      </c>
-      <c r="G1" s="3" t="s">
-        <v>19</v>
-      </c>
-      <c r="H1" s="3" t="s">
-        <v>20</v>
-      </c>
-      <c r="I1" s="3" t="s">
-        <v>21</v>
-      </c>
-      <c r="J1" s="3" t="s">
-        <v>22</v>
-      </c>
-      <c r="K1" s="3" t="s">
-        <v>23</v>
-      </c>
-      <c r="L1" s="3" t="s">
-        <v>24</v>
-      </c>
-      <c r="M1" s="3" t="s">
-        <v>31</v>
       </c>
     </row>
     <row r="2" spans="1:13" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
@@ -3667,7 +3680,7 @@
         <v>0</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>37</v>
+        <v>20</v>
       </c>
       <c r="C2" s="2">
         <v>0</v>
@@ -3676,16 +3689,16 @@
         <v>0</v>
       </c>
       <c r="E2" s="4" t="s">
-        <v>38</v>
+        <v>21</v>
       </c>
       <c r="F2" s="4" t="s">
-        <v>38</v>
+        <v>21</v>
       </c>
       <c r="G2" s="1" t="s">
-        <v>37</v>
+        <v>20</v>
       </c>
       <c r="H2" s="1" t="s">
-        <v>37</v>
+        <v>20</v>
       </c>
       <c r="I2" s="1"/>
       <c r="J2" s="3" t="b">
@@ -4570,11 +4583,11 @@
     <dataValidation type="list" allowBlank="1" showErrorMessage="1" errorTitle="Invalid Value" error="Please choose an option from the dropdown list." sqref="D2:D1048576 J2:M1048576" xr:uid="{4BB7CE7C-18FC-BB40-9E15-025F5FDB5F2D}">
       <formula1>"True, False"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showErrorMessage="1" errorTitle="Invalid Value" error="Please choose an option from the dropdown list." sqref="B2:B1048576" xr:uid="{04E1F09C-E3CF-9344-AD18-370A7D398746}">
-      <formula1>"context, public_question, private_question, discussion"</formula1>
-    </dataValidation>
     <dataValidation type="list" allowBlank="1" showErrorMessage="1" errorTitle="Invalid Value" error="Please choose an option from the dropdown list." sqref="H2:H1048576" xr:uid="{0624D554-C3E6-4644-B7AB-8913CD4B4670}">
       <formula1>"context, category, integer, free-text"</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showErrorMessage="1" errorTitle="Invalid Value" error="Please choose an option from the dropdown list." sqref="B2:B1048576" xr:uid="{411ACE32-59DA-9A46-8E0A-D56EB0BFB3B6}">
+      <formula1>"context, discussion, public_question, repeat_public_question, private_question, repeat_private_question"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0" footer="0"/>
@@ -4584,7 +4597,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
-  <dimension ref="C2:C5312"/>
+  <dimension ref="A1:C5312"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="11.1640625" defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="2" width="10.5" customWidth="1"/>
@@ -4594,47 +4607,56 @@
     <col min="22" max="41" width="10.5" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="3:3" s="6" customFormat="1" ht="16" x14ac:dyDescent="0.2"/>
-    <row r="3" spans="3:3" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A1" s="3" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" s="6" customFormat="1" ht="17" x14ac:dyDescent="0.2">
+      <c r="A2" s="7" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="C3" s="5"/>
     </row>
-    <row r="4" spans="3:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="C4" s="5"/>
     </row>
-    <row r="5" spans="3:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="C5" s="5"/>
     </row>
-    <row r="6" spans="3:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="C6" s="5"/>
     </row>
-    <row r="7" spans="3:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="C7" s="5"/>
     </row>
-    <row r="8" spans="3:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="C8" s="5"/>
     </row>
-    <row r="9" spans="3:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="C9" s="5"/>
     </row>
-    <row r="10" spans="3:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="C10" s="5"/>
     </row>
-    <row r="11" spans="3:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="C11" s="5"/>
     </row>
-    <row r="12" spans="3:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="C12" s="5"/>
     </row>
-    <row r="13" spans="3:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="C13" s="5"/>
     </row>
-    <row r="14" spans="3:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="C14" s="5"/>
     </row>
-    <row r="15" spans="3:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="C15" s="5"/>
     </row>
-    <row r="16" spans="3:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="C16" s="5"/>
     </row>
     <row r="17" spans="3:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
@@ -20547,10 +20569,10 @@
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
-        <v>25</v>
+        <v>32</v>
       </c>
       <c r="B1" s="3" t="s">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Fixed all remaining bugs in code and prompt template, improve format of output results in CSV format, and including experimental results from demo examples.
</commit_message>
<xml_diff>
--- a/demos/prompt_template.xlsx
+++ b/demos/prompt_template.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/raymondlow/Documents/talking-to-machines/talking-to-machines/demos/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AAC41F47-255B-584E-9FD4-DC9AE09E0AC3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A3D6639F-19EB-9349-813B-E635659020DD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="3620" yWindow="3400" windowWidth="34560" windowHeight="20140" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="3620" yWindow="3400" windowWidth="34560" windowHeight="20140" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="settings" sheetId="1" r:id="rId1"/>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="46" uniqueCount="40">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="48" uniqueCount="42">
   <si>
     <t>value</t>
   </si>
@@ -155,6 +155,14 @@
   </si>
   <si>
     <t>max_num_rounds</t>
+  </si>
+  <si>
+    <t>treatment</t>
+  </si>
+  <si>
+    <t>{
+"description":"This is the description of your treatment arm."
+}</t>
   </si>
 </sst>
 </file>
@@ -1572,8 +1580,12 @@
       </c>
     </row>
     <row r="2" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A2" s="1"/>
-      <c r="B2" s="1"/>
+      <c r="A2" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="B2" s="4" t="s">
+        <v>41</v>
+      </c>
     </row>
     <row r="3" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A3" s="1"/>

</xml_diff>